<commit_message>
Address review: add debt service to cash flow, align operating-day narrative
Codex review on PR #2:
- Cash flow now includes loan interest and principal repayment as
  Year-1 cash outflows (new "Срок кредита (лет)" assumption, straight-line
  paydown consistent with the declining P&L interest). Added a memo line
  for accrued Corporation Tax, noting it is paid in Year 2 (9 months after
  the accounting period ends), so it is correctly outside the Year-1 net
  flow. Year-1 ending cash stays positive (~£19k) after debt service.
- Aligned the operating-schedule wording in README, business plan (md +
  docx) with the model: ~7 days/week ≈ 332 operating days/year (with
  holidays/closures), not 365 — removing the ~£285k vs ~£312k discrepancy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PetgqhPEPFmBEho5MNCqhp
</commit_message>
<xml_diff>
--- a/shawarma-london/Финансовая_модель.xlsx
+++ b/shawarma-london/Финансовая_модель.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Инструкция" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Допущения" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Меню и фудкост" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Выручка" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Персонал" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Опер. расходы" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Стартовые вложения" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="P&amp;L (3 года)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Cash flow" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Безубыточность" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Налоги" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Допущения" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Меню и фудкост" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Выручка" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Персонал" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Опер. расходы" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Стартовые вложения" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L (3 года)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash flow" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Безубыточность" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Налоги" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -192,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -296,6 +296,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -924,7 +930,7 @@
           <t>Маржинальный доход на заказ</t>
         </is>
       </c>
-      <c r="B5" s="40">
+      <c r="B5" s="42">
         <f>B3-B4</f>
         <v/>
       </c>
@@ -974,7 +980,7 @@
           <t>Точка безубыточности (заказов/день)</t>
         </is>
       </c>
-      <c r="B8" s="41">
+      <c r="B8" s="43">
         <f>B7/'Выручка'!$O$4</f>
         <v/>
       </c>
@@ -1006,7 +1012,7 @@
           <t>Запас прочности</t>
         </is>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="44">
         <f>('Допущения'!$B$5-B8)/'Допущения'!$B$5</f>
         <v/>
       </c>
@@ -2204,6 +2210,26 @@
       <c r="D47" s="10" t="inlineStr">
         <is>
           <t>Ориентир.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>Срок кредита (лет)</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>лет</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Равномерное погашение тела; проценты убывают.</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4698,7 +4724,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Мес.0 — запуск (CapEx, финансирование). НДС уплачивается поквартально.</t>
+          <t>Мес.0 — запуск (CapEx, финансирование). Включены обслуживание кредита (проценты+тело) и квартальный НДС.</t>
         </is>
       </c>
     </row>
@@ -5256,50 +5282,58 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>НДС к уплате (квартально)</t>
+          <t>Проценты по кредиту</t>
         </is>
       </c>
       <c r="B12" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <v>0</v>
+      <c r="C12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="D12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
       </c>
       <c r="E12" s="33">
-        <f>-(('Выручка'!C10+'Выручка'!D10+'Выручка'!E10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
-        <v/>
-      </c>
-      <c r="F12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="33" t="n">
-        <v>0</v>
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="F12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="G12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
       </c>
       <c r="H12" s="33">
-        <f>-(('Выручка'!F10+'Выручка'!G10+'Выручка'!H10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
-        <v/>
-      </c>
-      <c r="I12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="33" t="n">
-        <v>0</v>
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="I12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="J12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
       </c>
       <c r="K12" s="33">
-        <f>-(('Выручка'!I10+'Выручка'!J10+'Выручка'!K10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
-        <v/>
-      </c>
-      <c r="L12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="33" t="n">
-        <v>0</v>
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="L12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
+      </c>
+      <c r="M12" s="33">
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
+        <v/>
       </c>
       <c r="N12" s="33">
-        <f>-(('Выручка'!L10+'Выручка'!M10+'Выручка'!N10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
+        <f>-'Допущения'!$B$46*'Допущения'!$B$47/12</f>
         <v/>
       </c>
       <c r="O12" s="33">
@@ -5308,130 +5342,263 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Погашение тела кредита</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="D13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="E13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="F13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="G13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="H13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="I13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="J13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="K13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="L13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="M13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="N13" s="33">
+        <f>-'Допущения'!$B$46/'Допущения'!$B$48/12</f>
+        <v/>
+      </c>
+      <c r="O13" s="33">
+        <f>B13+SUM(C13:N13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>НДС к уплате (квартально)</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="33">
+        <f>-(('Выручка'!C10+'Выручка'!D10+'Выручка'!E10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
+        <v/>
+      </c>
+      <c r="F14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="33">
+        <f>-(('Выручка'!F10+'Выручка'!G10+'Выручка'!H10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
+        <v/>
+      </c>
+      <c r="I14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="33">
+        <f>-(('Выручка'!I10+'Выручка'!J10+'Выручка'!K10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="33">
+        <f>-(('Выручка'!L10+'Выручка'!M10+'Выручка'!N10)-('Опер. расходы'!$C$17/12*3*'Допущения'!$B$7/(1+'Допущения'!$B$7)))</f>
+        <v/>
+      </c>
+      <c r="O14" s="33">
+        <f>B14+SUM(C14:N14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Чистый денежный поток</t>
         </is>
       </c>
-      <c r="B13" s="34">
-        <f>SUM(B4:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="34">
-        <f>SUM(C4:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="34">
-        <f>SUM(D4:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="34">
-        <f>SUM(E4:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="34">
-        <f>SUM(F4:F12)</f>
-        <v/>
-      </c>
-      <c r="G13" s="34">
-        <f>SUM(G4:G12)</f>
-        <v/>
-      </c>
-      <c r="H13" s="34">
-        <f>SUM(H4:H12)</f>
-        <v/>
-      </c>
-      <c r="I13" s="34">
-        <f>SUM(I4:I12)</f>
-        <v/>
-      </c>
-      <c r="J13" s="34">
-        <f>SUM(J4:J12)</f>
-        <v/>
-      </c>
-      <c r="K13" s="34">
-        <f>SUM(K4:K12)</f>
-        <v/>
-      </c>
-      <c r="L13" s="34">
-        <f>SUM(L4:L12)</f>
-        <v/>
-      </c>
-      <c r="M13" s="34">
-        <f>SUM(M4:M12)</f>
-        <v/>
-      </c>
-      <c r="N13" s="34">
-        <f>SUM(N4:N12)</f>
-        <v/>
-      </c>
-      <c r="O13" s="34">
-        <f>B13+SUM(C13:N13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="B15" s="34">
+        <f>SUM(B4:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="34">
+        <f>SUM(C4:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="34">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="34">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="34">
+        <f>SUM(F4:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="34">
+        <f>SUM(G4:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="34">
+        <f>SUM(H4:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="34">
+        <f>SUM(I4:I14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="34">
+        <f>SUM(J4:J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="34">
+        <f>SUM(K4:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="34">
+        <f>SUM(L4:L14)</f>
+        <v/>
+      </c>
+      <c r="M15" s="34">
+        <f>SUM(M4:M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="34">
+        <f>SUM(N4:N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="34">
+        <f>B15+SUM(C15:N15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Остаток денежных средств (накопл.)</t>
         </is>
       </c>
-      <c r="B14" s="39">
-        <f>B13</f>
-        <v/>
-      </c>
-      <c r="C14" s="39">
-        <f>B14+C13</f>
-        <v/>
-      </c>
-      <c r="D14" s="39">
-        <f>C14+D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="39">
-        <f>D14+E13</f>
-        <v/>
-      </c>
-      <c r="F14" s="39">
-        <f>E14+F13</f>
-        <v/>
-      </c>
-      <c r="G14" s="39">
-        <f>F14+G13</f>
-        <v/>
-      </c>
-      <c r="H14" s="39">
-        <f>G14+H13</f>
-        <v/>
-      </c>
-      <c r="I14" s="39">
-        <f>H14+I13</f>
-        <v/>
-      </c>
-      <c r="J14" s="39">
-        <f>I14+J13</f>
-        <v/>
-      </c>
-      <c r="K14" s="39">
-        <f>J14+K13</f>
-        <v/>
-      </c>
-      <c r="L14" s="39">
-        <f>K14+L13</f>
-        <v/>
-      </c>
-      <c r="M14" s="39">
-        <f>L14+M13</f>
-        <v/>
-      </c>
-      <c r="N14" s="39">
-        <f>M14+N13</f>
-        <v/>
+      <c r="B16" s="39">
+        <f>B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="39">
+        <f>B16+C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="39">
+        <f>C16+D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="39">
+        <f>D16+E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="39">
+        <f>E16+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="39">
+        <f>F16+G15</f>
+        <v/>
+      </c>
+      <c r="H16" s="39">
+        <f>G16+H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="39">
+        <f>H16+I15</f>
+        <v/>
+      </c>
+      <c r="J16" s="39">
+        <f>I16+J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="39">
+        <f>J16+K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="39">
+        <f>K16+L15</f>
+        <v/>
+      </c>
+      <c r="M16" s="39">
+        <f>L16+M15</f>
+        <v/>
+      </c>
+      <c r="N16" s="39">
+        <f>M16+N15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Справка: Corporation tax начислен</t>
+        </is>
+      </c>
+      <c r="B18" s="40">
+        <f>-'P&amp;L (3 года)'!$B$18</f>
+        <v/>
+      </c>
+      <c r="C18" s="41" t="inlineStr">
+        <is>
+          <t>Не входит в поток Года 1: CT уплачивается через 9 мес + 1 день после конца отчётного года (т.е. в Год 2).</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
+    <mergeCell ref="C18:O18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>